<commit_message>
hopefully final sim update
</commit_message>
<xml_diff>
--- a/contaminated_lognormal_final_summary.xlsx
+++ b/contaminated_lognormal_final_summary.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user-pc\OneDrive\Documents\RP\Contaminated-log-normal-model-of-household-income-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DEA0C92-8769-46CE-B53D-5E54D9F43997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F98806-06EC-4424-95BE-653C422BF7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" r:id="rId1"/>
+    <sheet name="diagnostics" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>n</t>
   </si>
@@ -67,25 +68,55 @@
     <t>epsilon_mse</t>
   </si>
   <si>
-    <t>AIC_single</t>
-  </si>
-  <si>
-    <t>AIC_mix_reg</t>
-  </si>
-  <si>
-    <t>AIC_mix_mode</t>
-  </si>
-  <si>
-    <t>best_model</t>
-  </si>
-  <si>
-    <t>single</t>
-  </si>
-  <si>
-    <t>mix_reg</t>
-  </si>
-  <si>
-    <t>mix_mode</t>
+    <t>conv_rate_reg</t>
+  </si>
+  <si>
+    <t>conv_rate_mode</t>
+  </si>
+  <si>
+    <t>aic_win_single</t>
+  </si>
+  <si>
+    <t>aic_win_mix_reg</t>
+  </si>
+  <si>
+    <t>aic_win_mix_mode</t>
+  </si>
+  <si>
+    <t>bic_win_single</t>
+  </si>
+  <si>
+    <t>bic_win_mix_reg</t>
+  </si>
+  <si>
+    <t>bic_win_mix_mode</t>
+  </si>
+  <si>
+    <t>n_valid_gap</t>
+  </si>
+  <si>
+    <t>mean_logLik_gap</t>
+  </si>
+  <si>
+    <t>min_logLik_gap</t>
+  </si>
+  <si>
+    <t>max_logLik_gap</t>
+  </si>
+  <si>
+    <t>mean_abs_logLik_gap</t>
+  </si>
+  <si>
+    <t>prop_gap_gt_small</t>
+  </si>
+  <si>
+    <t>prop_gap_gt_large</t>
+  </si>
+  <si>
+    <t>n_reg_better_reps</t>
+  </si>
+  <si>
+    <t>n_mode_better_reps</t>
   </si>
 </sst>
 </file>
@@ -438,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -455,13 +486,17 @@
     <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -519,8 +554,20 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>100</v>
       </c>
@@ -531,55 +578,67 @@
         <v>0.6</v>
       </c>
       <c r="D2">
-        <v>2.0142000000000002</v>
+        <v>2.0184000000000002</v>
       </c>
       <c r="E2">
-        <v>1.4200000000000001E-2</v>
+        <v>1.84E-2</v>
       </c>
       <c r="F2">
-        <v>1.9699999999999999E-2</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="G2">
-        <v>0.50749999999999995</v>
+        <v>0.50409999999999999</v>
       </c>
       <c r="H2">
-        <v>7.4999999999999997E-3</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="I2">
-        <v>7.1000000000000004E-3</v>
+        <v>6.7999999999999996E-3</v>
       </c>
       <c r="J2">
-        <v>2.2791000000000001</v>
+        <v>2.3599000000000001</v>
       </c>
       <c r="K2">
-        <v>0.27910000000000001</v>
+        <v>0.3599</v>
       </c>
       <c r="L2">
-        <v>1.6224000000000001</v>
+        <v>1.4926999999999999</v>
       </c>
       <c r="M2">
-        <v>0.73680000000000001</v>
+        <v>0.72399999999999998</v>
       </c>
       <c r="N2">
-        <v>0.1368</v>
+        <v>0.124</v>
       </c>
       <c r="O2">
-        <v>6.25E-2</v>
+        <v>5.8099999999999999E-2</v>
       </c>
       <c r="P2">
-        <v>393.26920000000001</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>395.2937</v>
+        <v>1</v>
       </c>
       <c r="R2">
-        <v>395.2937</v>
-      </c>
-      <c r="S2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.81599999999999995</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>100</v>
       </c>
@@ -590,55 +649,67 @@
         <v>0.9</v>
       </c>
       <c r="D3">
-        <v>2.0182000000000002</v>
+        <v>2.0211000000000001</v>
       </c>
       <c r="E3">
-        <v>1.8200000000000001E-2</v>
+        <v>2.1100000000000001E-2</v>
       </c>
       <c r="F3">
-        <v>1.7100000000000001E-2</v>
+        <v>1.7299999999999999E-2</v>
       </c>
       <c r="G3">
-        <v>0.46850000000000003</v>
+        <v>0.47070000000000001</v>
       </c>
       <c r="H3">
-        <v>-3.15E-2</v>
+        <v>-2.93E-2</v>
       </c>
       <c r="I3">
-        <v>5.8999999999999999E-3</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="J3">
-        <v>2.1171000000000002</v>
+        <v>2.0708000000000002</v>
       </c>
       <c r="K3">
-        <v>0.1171</v>
+        <v>7.0800000000000002E-2</v>
       </c>
       <c r="L3">
-        <v>1.6696</v>
+        <v>1.5526</v>
       </c>
       <c r="M3">
-        <v>0.79310000000000003</v>
+        <v>0.79720000000000002</v>
       </c>
       <c r="N3">
-        <v>-0.1069</v>
+        <v>-0.1028</v>
       </c>
       <c r="O3">
-        <v>5.4399999999999997E-2</v>
+        <v>5.1499999999999997E-2</v>
       </c>
       <c r="P3">
-        <v>352.93340000000001</v>
+        <v>1</v>
       </c>
       <c r="Q3">
-        <v>355.37799999999999</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>355.37810000000002</v>
-      </c>
-      <c r="S3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.872</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0.97399999999999998</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>100</v>
       </c>
@@ -649,13 +720,13 @@
         <v>0.6</v>
       </c>
       <c r="D4">
-        <v>2.0162</v>
+        <v>2.0043000000000002</v>
       </c>
       <c r="E4">
-        <v>1.6199999999999999E-2</v>
+        <v>4.3E-3</v>
       </c>
       <c r="F4">
-        <v>2.9600000000000001E-2</v>
+        <v>3.3799999999999997E-2</v>
       </c>
       <c r="G4">
         <v>0.49740000000000001</v>
@@ -664,40 +735,52 @@
         <v>-2.5999999999999999E-3</v>
       </c>
       <c r="I4">
-        <v>7.6E-3</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="J4">
-        <v>5.5407000000000002</v>
+        <v>5.4942000000000002</v>
       </c>
       <c r="K4">
-        <v>0.54069999999999996</v>
+        <v>0.49419999999999997</v>
       </c>
       <c r="L4">
-        <v>3.1052</v>
+        <v>3.2581000000000002</v>
       </c>
       <c r="M4">
-        <v>0.6139</v>
+        <v>0.60799999999999998</v>
       </c>
       <c r="N4">
-        <v>1.3899999999999999E-2</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="O4">
-        <v>1.12E-2</v>
+        <v>1.0500000000000001E-2</v>
       </c>
       <c r="P4">
-        <v>543.33889999999997</v>
+        <v>1</v>
       </c>
       <c r="Q4">
-        <v>528.24890000000005</v>
+        <v>1</v>
       </c>
       <c r="R4">
-        <v>528.24890000000005</v>
-      </c>
-      <c r="S4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0.13400000000000001</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>100</v>
       </c>
@@ -708,55 +791,67 @@
         <v>0.9</v>
       </c>
       <c r="D5">
-        <v>2.0169999999999999</v>
+        <v>2.0049999999999999</v>
       </c>
       <c r="E5">
-        <v>1.7000000000000001E-2</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="F5">
-        <v>1.7399999999999999E-2</v>
+        <v>1.84E-2</v>
       </c>
       <c r="G5">
-        <v>0.47889999999999999</v>
+        <v>0.47849999999999998</v>
       </c>
       <c r="H5">
-        <v>-2.1100000000000001E-2</v>
+        <v>-2.1499999999999998E-2</v>
       </c>
       <c r="I5">
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="J5">
-        <v>5.3150000000000004</v>
+        <v>5.3390000000000004</v>
       </c>
       <c r="K5">
-        <v>0.315</v>
+        <v>0.33900000000000002</v>
       </c>
       <c r="L5">
-        <v>3.5225</v>
+        <v>3.7178</v>
       </c>
       <c r="M5">
-        <v>0.84489999999999998</v>
+        <v>0.85089999999999999</v>
       </c>
       <c r="N5">
-        <v>-5.5100000000000003E-2</v>
+        <v>-4.9099999999999998E-2</v>
       </c>
       <c r="O5">
-        <v>1.77E-2</v>
+        <v>1.6E-2</v>
       </c>
       <c r="P5">
-        <v>413.62959999999998</v>
+        <v>1</v>
       </c>
       <c r="Q5">
-        <v>399.17320000000001</v>
+        <v>1</v>
       </c>
       <c r="R5">
-        <v>399.17340000000002</v>
-      </c>
-      <c r="S5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.09</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0.22600000000000001</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1000</v>
       </c>
@@ -767,55 +862,67 @@
         <v>0.6</v>
       </c>
       <c r="D6">
-        <v>2.0013000000000001</v>
+        <v>2.0013999999999998</v>
       </c>
       <c r="E6">
-        <v>1.2999999999999999E-3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="F6">
         <v>2E-3</v>
       </c>
       <c r="G6">
-        <v>0.50560000000000005</v>
+        <v>0.50449999999999995</v>
       </c>
       <c r="H6">
-        <v>5.5999999999999999E-3</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="I6">
         <v>1.5E-3</v>
       </c>
       <c r="J6">
-        <v>2.1366000000000001</v>
+        <v>2.1208999999999998</v>
       </c>
       <c r="K6">
-        <v>0.1366</v>
+        <v>0.12089999999999999</v>
       </c>
       <c r="L6">
-        <v>0.1547</v>
+        <v>0.1492</v>
       </c>
       <c r="M6">
-        <v>0.64710000000000001</v>
+        <v>0.63590000000000002</v>
       </c>
       <c r="N6">
-        <v>4.7100000000000003E-2</v>
+        <v>3.5900000000000001E-2</v>
       </c>
       <c r="O6">
-        <v>2.63E-2</v>
+        <v>2.47E-2</v>
       </c>
       <c r="P6">
-        <v>3916.5072</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>3908.9335000000001</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>3908.9335000000001</v>
-      </c>
-      <c r="S6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.152</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0.69</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -826,55 +933,67 @@
         <v>0.9</v>
       </c>
       <c r="D7">
-        <v>2.0001000000000002</v>
+        <v>2.0011000000000001</v>
       </c>
       <c r="E7">
-        <v>1E-4</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="F7">
-        <v>1.5E-3</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="G7">
-        <v>0.4854</v>
+        <v>0.48570000000000002</v>
       </c>
       <c r="H7">
-        <v>-1.46E-2</v>
+        <v>-1.43E-2</v>
       </c>
       <c r="I7">
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="J7">
-        <v>2.1848999999999998</v>
+        <v>2.1941999999999999</v>
       </c>
       <c r="K7">
-        <v>0.18490000000000001</v>
+        <v>0.19420000000000001</v>
       </c>
       <c r="L7">
-        <v>0.6452</v>
+        <v>0.69810000000000005</v>
       </c>
       <c r="M7">
-        <v>0.79220000000000002</v>
+        <v>0.79820000000000002</v>
       </c>
       <c r="N7">
-        <v>-0.10780000000000001</v>
+        <v>-0.1018</v>
       </c>
       <c r="O7">
-        <v>4.6699999999999998E-2</v>
+        <v>4.5400000000000003E-2</v>
       </c>
       <c r="P7">
-        <v>3501.5716000000002</v>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <v>3499.4733000000001</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>3499.4733999999999</v>
-      </c>
-      <c r="S7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.442</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1000</v>
       </c>
@@ -885,55 +1004,67 @@
         <v>0.6</v>
       </c>
       <c r="D8">
-        <v>2.0001000000000002</v>
+        <v>2.0011000000000001</v>
       </c>
       <c r="E8">
-        <v>1E-4</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="F8">
-        <v>2.7000000000000001E-3</v>
+        <v>2.8E-3</v>
       </c>
       <c r="G8">
-        <v>0.49859999999999999</v>
+        <v>0.49919999999999998</v>
       </c>
       <c r="H8">
-        <v>-1.4E-3</v>
+        <v>-8.0000000000000004E-4</v>
       </c>
       <c r="I8">
         <v>6.9999999999999999E-4</v>
       </c>
       <c r="J8">
-        <v>5.0667</v>
+        <v>5.0603999999999996</v>
       </c>
       <c r="K8">
-        <v>6.6699999999999995E-2</v>
+        <v>6.0400000000000002E-2</v>
       </c>
       <c r="L8">
-        <v>0.22189999999999999</v>
+        <v>0.2198</v>
       </c>
       <c r="M8">
-        <v>0.60089999999999999</v>
+        <v>0.60140000000000005</v>
       </c>
       <c r="N8">
-        <v>8.9999999999999998E-4</v>
+        <v>1.4E-3</v>
       </c>
       <c r="O8">
         <v>1.6000000000000001E-3</v>
       </c>
       <c r="P8">
-        <v>5405.5736999999999</v>
+        <v>1</v>
       </c>
       <c r="Q8">
-        <v>5231.1899000000003</v>
+        <v>1</v>
       </c>
       <c r="R8">
-        <v>5231.1899000000003</v>
-      </c>
-      <c r="S8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -944,55 +1075,67 @@
         <v>0.9</v>
       </c>
       <c r="D9">
-        <v>2.0015000000000001</v>
+        <v>2.0013000000000001</v>
       </c>
       <c r="E9">
-        <v>1.5E-3</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="F9">
         <v>1.8E-3</v>
       </c>
       <c r="G9">
-        <v>0.49840000000000001</v>
+        <v>0.49809999999999999</v>
       </c>
       <c r="H9">
-        <v>-1.6000000000000001E-3</v>
+        <v>-1.9E-3</v>
       </c>
       <c r="I9">
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="J9">
-        <v>5.0381</v>
+        <v>5.0483000000000002</v>
       </c>
       <c r="K9">
-        <v>3.8100000000000002E-2</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="L9">
-        <v>0.32079999999999997</v>
+        <v>0.31090000000000001</v>
       </c>
       <c r="M9">
-        <v>0.89610000000000001</v>
+        <v>0.89600000000000002</v>
       </c>
       <c r="N9">
-        <v>-3.8999999999999998E-3</v>
+        <v>-4.0000000000000001E-3</v>
       </c>
       <c r="O9">
         <v>5.9999999999999995E-4</v>
       </c>
       <c r="P9">
-        <v>4109.8957</v>
+        <v>1</v>
       </c>
       <c r="Q9">
-        <v>3938.2438999999999</v>
+        <v>1</v>
       </c>
       <c r="R9">
-        <v>3938.2438999999999</v>
-      </c>
-      <c r="S9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10000</v>
       </c>
@@ -1003,55 +1146,67 @@
         <v>0.6</v>
       </c>
       <c r="D10">
-        <v>1.9995000000000001</v>
+        <v>1.9994000000000001</v>
       </c>
       <c r="E10">
-        <v>-5.0000000000000001E-4</v>
+        <v>-5.9999999999999995E-4</v>
       </c>
       <c r="F10">
         <v>2.0000000000000001E-4</v>
       </c>
       <c r="G10">
-        <v>0.49919999999999998</v>
+        <v>0.4995</v>
       </c>
       <c r="H10">
-        <v>-8.0000000000000004E-4</v>
+        <v>-5.0000000000000001E-4</v>
       </c>
       <c r="I10">
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="J10">
-        <v>2.0249999999999999</v>
+        <v>2.0270000000000001</v>
       </c>
       <c r="K10">
-        <v>2.5000000000000001E-2</v>
+        <v>2.7E-2</v>
       </c>
       <c r="L10">
         <v>8.5000000000000006E-3</v>
       </c>
       <c r="M10">
-        <v>0.60150000000000003</v>
+        <v>0.60329999999999995</v>
       </c>
       <c r="N10">
-        <v>1.5E-3</v>
+        <v>3.3E-3</v>
       </c>
       <c r="O10">
-        <v>6.4000000000000003E-3</v>
+        <v>6.8999999999999999E-3</v>
       </c>
       <c r="P10">
-        <v>39167.609700000001</v>
+        <v>1</v>
       </c>
       <c r="Q10">
-        <v>39070.726799999997</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>39070.726799999997</v>
-      </c>
-      <c r="S10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10000</v>
       </c>
@@ -1062,55 +1217,67 @@
         <v>0.9</v>
       </c>
       <c r="D11">
-        <v>2.0005000000000002</v>
+        <v>2.0003000000000002</v>
       </c>
       <c r="E11">
-        <v>5.0000000000000001E-4</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="F11">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="G11">
+        <v>0.49719999999999998</v>
+      </c>
+      <c r="H11">
+        <v>-2.8E-3</v>
+      </c>
+      <c r="I11">
         <v>1E-4</v>
       </c>
-      <c r="G11">
-        <v>0.49669999999999997</v>
-      </c>
-      <c r="H11">
-        <v>-3.3E-3</v>
-      </c>
-      <c r="I11">
-        <v>2.0000000000000001E-4</v>
-      </c>
       <c r="J11">
-        <v>2.0297999999999998</v>
+        <v>2.0356999999999998</v>
       </c>
       <c r="K11">
-        <v>2.98E-2</v>
+        <v>3.5700000000000003E-2</v>
       </c>
       <c r="L11">
-        <v>6.2300000000000001E-2</v>
+        <v>5.8599999999999999E-2</v>
       </c>
       <c r="M11">
-        <v>0.87019999999999997</v>
+        <v>0.87529999999999997</v>
       </c>
       <c r="N11">
-        <v>-2.98E-2</v>
+        <v>-2.47E-2</v>
       </c>
       <c r="O11">
-        <v>9.1999999999999998E-3</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="P11">
-        <v>35042.457199999997</v>
+        <v>1</v>
       </c>
       <c r="Q11">
-        <v>35000.406600000002</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>35000.406600000002</v>
-      </c>
-      <c r="S11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0.02</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10000</v>
       </c>
@@ -1121,55 +1288,67 @@
         <v>0.6</v>
       </c>
       <c r="D12">
-        <v>1.9997</v>
+        <v>2.0001000000000002</v>
       </c>
       <c r="E12">
-        <v>-2.9999999999999997E-4</v>
+        <v>1E-4</v>
       </c>
       <c r="F12">
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="G12">
-        <v>0.49990000000000001</v>
+        <v>0.50049999999999994</v>
       </c>
       <c r="H12">
-        <v>-1E-4</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I12">
         <v>1E-4</v>
       </c>
       <c r="J12">
-        <v>5.0058999999999996</v>
+        <v>5.0007000000000001</v>
       </c>
       <c r="K12">
-        <v>5.8999999999999999E-3</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="L12">
-        <v>2.1000000000000001E-2</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="M12">
-        <v>0.59960000000000002</v>
+        <v>0.60070000000000001</v>
       </c>
       <c r="N12">
-        <v>-4.0000000000000002E-4</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="O12">
         <v>2.0000000000000001E-4</v>
       </c>
       <c r="P12">
-        <v>54091.459900000002</v>
+        <v>1</v>
       </c>
       <c r="Q12">
-        <v>52334.689700000003</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>52334.689700000003</v>
-      </c>
-      <c r="S12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10000</v>
       </c>
@@ -1180,52 +1359,580 @@
         <v>0.9</v>
       </c>
       <c r="D13">
-        <v>2.0004</v>
+        <v>2.0005000000000002</v>
       </c>
       <c r="E13">
-        <v>4.0000000000000002E-4</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="F13">
         <v>2.0000000000000001E-4</v>
       </c>
       <c r="G13">
-        <v>0.5</v>
+        <v>0.49990000000000001</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>-1E-4</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13">
-        <v>5.0033000000000003</v>
+        <v>4.9970999999999997</v>
       </c>
       <c r="K13">
-        <v>3.3E-3</v>
+        <v>-2.8999999999999998E-3</v>
       </c>
       <c r="L13">
-        <v>3.0800000000000001E-2</v>
+        <v>3.2500000000000001E-2</v>
       </c>
       <c r="M13">
-        <v>0.89959999999999996</v>
+        <v>0.89929999999999999</v>
       </c>
       <c r="N13">
-        <v>-4.0000000000000002E-4</v>
+        <v>-6.9999999999999999E-4</v>
       </c>
       <c r="O13">
         <v>1E-4</v>
       </c>
       <c r="P13">
-        <v>41050.698799999998</v>
+        <v>1</v>
       </c>
       <c r="Q13">
-        <v>39318.336000000003</v>
+        <v>1</v>
       </c>
       <c r="R13">
-        <v>39318.336000000003</v>
-      </c>
-      <c r="S13" t="s">
-        <v>21</v>
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>100</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>0.6</v>
+      </c>
+      <c r="D2">
+        <v>500</v>
+      </c>
+      <c r="E2">
+        <v>-2.0000000000000002E-5</v>
+      </c>
+      <c r="F2">
+        <v>-5.5199999999999997E-3</v>
+      </c>
+      <c r="G2">
+        <v>2.8400000000000001E-3</v>
+      </c>
+      <c r="H2">
+        <v>4.0000000000000003E-5</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>246</v>
+      </c>
+      <c r="L2">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>100</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>0.9</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+      <c r="E3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="F3">
+        <v>-9.8999999999999999E-4</v>
+      </c>
+      <c r="G3">
+        <v>3.9399999999999999E-3</v>
+      </c>
+      <c r="H3">
+        <v>2.0000000000000002E-5</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>262</v>
+      </c>
+      <c r="L3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>100</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>0.6</v>
+      </c>
+      <c r="D4">
+        <v>500</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>245</v>
+      </c>
+      <c r="L4">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>100</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>0.9</v>
+      </c>
+      <c r="D5">
+        <v>500</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>255</v>
+      </c>
+      <c r="L5">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1000</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>0.6</v>
+      </c>
+      <c r="D6">
+        <v>500</v>
+      </c>
+      <c r="E6">
+        <v>6.0000000000000002E-5</v>
+      </c>
+      <c r="F6">
+        <v>-9.7000000000000005E-4</v>
+      </c>
+      <c r="G6">
+        <v>2.316E-2</v>
+      </c>
+      <c r="H6">
+        <v>8.0000000000000007E-5</v>
+      </c>
+      <c r="I6">
+        <v>2E-3</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>247</v>
+      </c>
+      <c r="L6">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>0.9</v>
+      </c>
+      <c r="D7">
+        <v>500</v>
+      </c>
+      <c r="E7">
+        <v>2.0000000000000002E-5</v>
+      </c>
+      <c r="F7">
+        <v>-5.1999999999999995E-4</v>
+      </c>
+      <c r="G7">
+        <v>2.14E-3</v>
+      </c>
+      <c r="H7">
+        <v>3.0000000000000001E-5</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>245</v>
+      </c>
+      <c r="L7">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1000</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>0.6</v>
+      </c>
+      <c r="D8">
+        <v>500</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>-2.0000000000000002E-5</v>
+      </c>
+      <c r="G8">
+        <v>5.0000000000000002E-5</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>255</v>
+      </c>
+      <c r="L8">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9">
+        <v>0.9</v>
+      </c>
+      <c r="D9">
+        <v>500</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>-1.0000000000000001E-5</v>
+      </c>
+      <c r="G9">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>256</v>
+      </c>
+      <c r="L9">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>10000</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>0.6</v>
+      </c>
+      <c r="D10">
+        <v>500</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>-2.8800000000000002E-3</v>
+      </c>
+      <c r="G10">
+        <v>3.8E-3</v>
+      </c>
+      <c r="H10">
+        <v>1E-4</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>267</v>
+      </c>
+      <c r="L10">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10000</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>0.9</v>
+      </c>
+      <c r="D11">
+        <v>500</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>-2.4000000000000001E-4</v>
+      </c>
+      <c r="G11">
+        <v>1.06E-3</v>
+      </c>
+      <c r="H11">
+        <v>4.0000000000000003E-5</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>229</v>
+      </c>
+      <c r="L11">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10000</v>
+      </c>
+      <c r="B12">
+        <v>5</v>
+      </c>
+      <c r="C12">
+        <v>0.6</v>
+      </c>
+      <c r="D12">
+        <v>500</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>-1.7000000000000001E-4</v>
+      </c>
+      <c r="G12">
+        <v>1.4999999999999999E-4</v>
+      </c>
+      <c r="H12">
+        <v>4.0000000000000003E-5</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>246</v>
+      </c>
+      <c r="L12">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>10000</v>
+      </c>
+      <c r="B13">
+        <v>5</v>
+      </c>
+      <c r="C13">
+        <v>0.9</v>
+      </c>
+      <c r="D13">
+        <v>500</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>-1.2E-4</v>
+      </c>
+      <c r="G13">
+        <v>1E-4</v>
+      </c>
+      <c r="H13">
+        <v>3.0000000000000001E-5</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>248</v>
+      </c>
+      <c r="L13">
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>